<commit_message>
fix: guild card click popup via pointerup, remove training simulator preview cards
</commit_message>
<xml_diff>
--- a/reports/빅딜/빅딜_league_mgf_report.xlsx
+++ b/reports/빅딜/빅딜_league_mgf_report.xlsx
@@ -18,7 +18,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">guilds!$A$1:$M$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">밤과다람쥐!$A$1:$J$29</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">부계둘!$A$1:$J$30</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">빅딜!$A$1:$J$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">빅딜!$A$1:$J$29</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">이고이스트!$A$1:$J$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">피난민!$A$1:$J$30</definedName>
   </definedNames>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1578" uniqueCount="560">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1568" uniqueCount="556">
   <si>
     <t>guild_name</t>
   </si>
@@ -254,7 +254,7 @@
     <t>103</t>
   </si>
   <si>
-    <t>15조 1221억 9952만</t>
+    <t>15조 2195억 3666만</t>
   </si>
   <si>
     <t>2</t>
@@ -272,57 +272,57 @@
     <t>신궁</t>
   </si>
   <si>
+    <t>14조 951억 2182만</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>킹몬</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%ED%82%B9%EB%AA%AC</t>
+  </si>
+  <si>
+    <t>다크나이트</t>
+  </si>
+  <si>
+    <t>100</t>
+  </si>
+  <si>
+    <t>12조 6365억 3160만</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>엘라임</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EC%97%98%EB%9D%BC%EC%9E%84</t>
+  </si>
+  <si>
+    <t>히어로</t>
+  </si>
+  <si>
+    <t>10조 7888억 6150만</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>야가다</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EC%95%BC%EA%B0%80%EB%8B%A4</t>
+  </si>
+  <si>
+    <t>보우마스터</t>
+  </si>
+  <si>
     <t>102</t>
   </si>
   <si>
-    <t>14조 951억 2182만</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>킹몬</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%ED%82%B9%EB%AA%AC</t>
-  </si>
-  <si>
-    <t>다크나이트</t>
-  </si>
-  <si>
-    <t>100</t>
-  </si>
-  <si>
-    <t>12조 6365억 3160만</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>엘라임</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EC%97%98%EB%9D%BC%EC%9E%84</t>
-  </si>
-  <si>
-    <t>히어로</t>
-  </si>
-  <si>
-    <t>10조 6714억 9011만</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t>야가다</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EC%95%BC%EA%B0%80%EB%8B%A4</t>
-  </si>
-  <si>
-    <t>보우마스터</t>
-  </si>
-  <si>
     <t>9조 4831억 8007만</t>
   </si>
   <si>
@@ -335,7 +335,7 @@
     <t>https://mgf.gg/contents/character.php?n=%EB%8B%A8%ED%92%8D%EC%B9%B4%EC%9A%B0</t>
   </si>
   <si>
-    <t>7조 3899억 9567만</t>
+    <t>8조 3534억 4319만</t>
   </si>
   <si>
     <t>7</t>
@@ -377,7 +377,7 @@
     <t>https://mgf.gg/contents/character.php?n=%ED%8F%AC%EC%8A%A4%EC%BD%94%ED%93%A8%EC%B2%98%EC%97%A0</t>
   </si>
   <si>
-    <t>5조 1472억 5810만</t>
+    <t>5조 1592억 3651만</t>
   </si>
   <si>
     <t>10</t>
@@ -407,7 +407,7 @@
     <t>https://mgf.gg/contents/character.php?n=%EC%9A%B0%ED%9B%84</t>
   </si>
   <si>
-    <t>3조 8750억 1931만</t>
+    <t>4조 2089억 9652만</t>
   </si>
   <si>
     <t>12</t>
@@ -449,6 +449,21 @@
     <t>15</t>
   </si>
   <si>
+    <t>비스밤</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EB%B9%84%EC%8A%A4%EB%B0%A4</t>
+  </si>
+  <si>
+    <t>98</t>
+  </si>
+  <si>
+    <t>2조 5943억 9545만</t>
+  </si>
+  <si>
+    <t>16</t>
+  </si>
+  <si>
     <t>아르젠타</t>
   </si>
   <si>
@@ -461,18 +476,6 @@
     <t>2조 5940억 8239만</t>
   </si>
   <si>
-    <t>16</t>
-  </si>
-  <si>
-    <t>비스밤</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EB%B9%84%EC%8A%A4%EB%B0%A4</t>
-  </si>
-  <si>
-    <t>2조 5711억 1705만</t>
-  </si>
-  <si>
     <t>17</t>
   </si>
   <si>
@@ -488,30 +491,27 @@
     <t>18</t>
   </si>
   <si>
+    <t>민들레꽃</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EB%AF%BC%EB%93%A4%EB%A0%88%EA%BD%83</t>
+  </si>
+  <si>
+    <t>2조 5359억 851만</t>
+  </si>
+  <si>
+    <t>19</t>
+  </si>
+  <si>
     <t>꾸르꾸르</t>
   </si>
   <si>
     <t>https://mgf.gg/contents/character.php?n=%EA%BE%B8%EB%A5%B4%EA%BE%B8%EB%A5%B4</t>
   </si>
   <si>
-    <t>98</t>
-  </si>
-  <si>
     <t>2조 3765억 8123만</t>
   </si>
   <si>
-    <t>19</t>
-  </si>
-  <si>
-    <t>민들레꽃</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EB%AF%BC%EB%93%A4%EB%A0%88%EA%BD%83</t>
-  </si>
-  <si>
-    <t>2조 3302억 2720만</t>
-  </si>
-  <si>
     <t>20</t>
   </si>
   <si>
@@ -578,6 +578,18 @@
     <t>25</t>
   </si>
   <si>
+    <t>데드캣</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EB%8D%B0%EB%93%9C%EC%BA%A3</t>
+  </si>
+  <si>
+    <t>1조 8260억 5446만</t>
+  </si>
+  <si>
+    <t>26</t>
+  </si>
+  <si>
     <t>여눈</t>
   </si>
   <si>
@@ -587,7 +599,7 @@
     <t>1조 7856억 5439만</t>
   </si>
   <si>
-    <t>26</t>
+    <t>27</t>
   </si>
   <si>
     <t>플로우00</t>
@@ -599,18 +611,6 @@
     <t>1조 6923억 5834만</t>
   </si>
   <si>
-    <t>27</t>
-  </si>
-  <si>
-    <t>데드캣</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EB%8D%B0%EB%93%9C%EC%BA%A3</t>
-  </si>
-  <si>
-    <t>1조 6435억 7464만</t>
-  </si>
-  <si>
     <t>28</t>
   </si>
   <si>
@@ -626,282 +626,270 @@
     <t>1조 2381억 1362만</t>
   </si>
   <si>
+    <t>증권보이</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EC%A6%9D%EA%B6%8C%EB%B3%B4%EC%9D%B4</t>
+  </si>
+  <si>
+    <t>20조 4898억 61만</t>
+  </si>
+  <si>
+    <t>둥둥콩이</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EB%91%A5%EB%91%A5%EC%BD%A9%EC%9D%B4</t>
+  </si>
+  <si>
+    <t>19조 9942억 330만</t>
+  </si>
+  <si>
+    <t>가온스</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EA%B0%80%EC%98%A8%EC%8A%A4</t>
+  </si>
+  <si>
+    <t>17조 4585억 7977만</t>
+  </si>
+  <si>
+    <t>Canary</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=Canary</t>
+  </si>
+  <si>
+    <t>15조 8193억 825만</t>
+  </si>
+  <si>
+    <t>처히</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EC%B2%98%ED%9E%88</t>
+  </si>
+  <si>
+    <t>13조 2156억 7422만</t>
+  </si>
+  <si>
+    <t>환생의불꼬츠</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%ED%99%98%EC%83%9D%EC%9D%98%EB%B6%88%EA%BC%AC%EC%B8%A0</t>
+  </si>
+  <si>
+    <t>10조 9549억 8302만</t>
+  </si>
+  <si>
+    <t>밍진</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EB%B0%8D%EC%A7%84</t>
+  </si>
+  <si>
+    <t>8조 9166억 6911만</t>
+  </si>
+  <si>
+    <t>Naco</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=Naco</t>
+  </si>
+  <si>
+    <t>6조 9849억 7135만</t>
+  </si>
+  <si>
+    <t>AKPS</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=AKPS</t>
+  </si>
+  <si>
+    <t>6조 5629억 7412만</t>
+  </si>
+  <si>
+    <t>사나이기백황</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EC%82%AC%EB%82%98%EC%9D%B4%EA%B8%B0%EB%B0%B1%ED%99%A9</t>
+  </si>
+  <si>
+    <t>3조 8303억 3845만</t>
+  </si>
+  <si>
+    <t>토미오카상</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%ED%86%A0%EB%AF%B8%EC%98%A4%EC%B9%B4%EC%83%81</t>
+  </si>
+  <si>
+    <t>3조 3002억 4541만</t>
+  </si>
+  <si>
+    <t>평평이형</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%ED%8F%89%ED%8F%89%EC%9D%B4%ED%98%95</t>
+  </si>
+  <si>
+    <t>3조 906억 3513만</t>
+  </si>
+  <si>
+    <t>천칠</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EC%B2%9C%EC%B9%A0</t>
+  </si>
+  <si>
+    <t>팔라딘</t>
+  </si>
+  <si>
+    <t>2조 6702억 2482만</t>
+  </si>
+  <si>
+    <t>토니워터</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%ED%86%A0%EB%8B%88%EC%9B%8C%ED%84%B0</t>
+  </si>
+  <si>
+    <t>2조 6162억 1545만</t>
+  </si>
+  <si>
+    <t>펑풀</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%ED%8E%91%ED%92%80</t>
+  </si>
+  <si>
+    <t>2조 4885억 7115만</t>
+  </si>
+  <si>
+    <t>화살대</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%ED%99%94%EC%82%B4%EB%8C%80</t>
+  </si>
+  <si>
+    <t>2조 4258억 6186만</t>
+  </si>
+  <si>
+    <t>런닝래빗</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EB%9F%B0%EB%8B%9D%EB%9E%98%EB%B9%97</t>
+  </si>
+  <si>
+    <t>2조 4177억 8071만</t>
+  </si>
+  <si>
+    <t>피어난</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%ED%94%BC%EC%96%B4%EB%82%9C</t>
+  </si>
+  <si>
+    <t>2조 305억 8537만</t>
+  </si>
+  <si>
+    <t>샤스찌에</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EC%83%A4%EC%8A%A4%EC%B0%8C%EC%97%90</t>
+  </si>
+  <si>
+    <t>1조 4976억 9640만</t>
+  </si>
+  <si>
+    <t>보동핑</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EB%B3%B4%EB%8F%99%ED%95%91</t>
+  </si>
+  <si>
+    <t>1조 1820억 5434만</t>
+  </si>
+  <si>
+    <t>싸토루</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EC%8B%B8%ED%86%A0%EB%A3%A8</t>
+  </si>
+  <si>
+    <t>95</t>
+  </si>
+  <si>
+    <t>1조 1480억 9108만</t>
+  </si>
+  <si>
+    <t>지니좋아요</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EC%A7%80%EB%8B%88%EC%A2%8B%EC%95%84%EC%9A%94</t>
+  </si>
+  <si>
+    <t>1조 666억 9786만</t>
+  </si>
+  <si>
+    <t>2026년1월30일</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=2026%EB%85%841%EC%9B%9430%EC%9D%BC</t>
+  </si>
+  <si>
+    <t>1조 129억 4198만</t>
+  </si>
+  <si>
+    <t>찐곽정근</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EC%B0%90%EA%B3%BD%EC%A0%95%EA%B7%BC</t>
+  </si>
+  <si>
+    <t>1조 24억 1640만</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%ED%99%8D%EC%B6%98%EC%82%BC</t>
+  </si>
+  <si>
+    <t>8747억 2403만</t>
+  </si>
+  <si>
+    <t>Targa</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=Targa</t>
+  </si>
+  <si>
+    <t>94</t>
+  </si>
+  <si>
+    <t>5665억 5826만</t>
+  </si>
+  <si>
+    <t>애둘이에요</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EC%95%A0%EB%91%98%EC%9D%B4%EC%97%90%EC%9A%94</t>
+  </si>
+  <si>
+    <t>93</t>
+  </si>
+  <si>
+    <t>5424억 3794만</t>
+  </si>
+  <si>
+    <t>짱창훈</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EC%A7%B1%EC%B0%BD%ED%9B%88</t>
+  </si>
+  <si>
+    <t>3382억 604만</t>
+  </si>
+  <si>
     <t>29</t>
   </si>
   <si>
-    <t>혜영인기도1</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%ED%98%9C%EC%98%81%EC%9D%B8%EA%B8%B0%EB%8F%841</t>
-  </si>
-  <si>
-    <t>76</t>
-  </si>
-  <si>
-    <t>11억 9359만</t>
-  </si>
-  <si>
-    <t>증권보이</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EC%A6%9D%EA%B6%8C%EB%B3%B4%EC%9D%B4</t>
-  </si>
-  <si>
-    <t>20조 4898억 61만</t>
-  </si>
-  <si>
-    <t>둥둥콩이</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EB%91%A5%EB%91%A5%EC%BD%A9%EC%9D%B4</t>
-  </si>
-  <si>
-    <t>19조 9942억 330만</t>
-  </si>
-  <si>
-    <t>가온스</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EA%B0%80%EC%98%A8%EC%8A%A4</t>
-  </si>
-  <si>
-    <t>17조 4585억 7977만</t>
-  </si>
-  <si>
-    <t>Canary</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=Canary</t>
-  </si>
-  <si>
-    <t>15조 8193억 825만</t>
-  </si>
-  <si>
-    <t>처히</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EC%B2%98%ED%9E%88</t>
-  </si>
-  <si>
-    <t>13조 2156억 7422만</t>
-  </si>
-  <si>
-    <t>환생의불꼬츠</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%ED%99%98%EC%83%9D%EC%9D%98%EB%B6%88%EA%BC%AC%EC%B8%A0</t>
-  </si>
-  <si>
-    <t>10조 9549억 8302만</t>
-  </si>
-  <si>
-    <t>밍진</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EB%B0%8D%EC%A7%84</t>
-  </si>
-  <si>
-    <t>8조 9166억 6911만</t>
-  </si>
-  <si>
-    <t>Naco</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=Naco</t>
-  </si>
-  <si>
-    <t>6조 9849억 7135만</t>
-  </si>
-  <si>
-    <t>AKPS</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=AKPS</t>
-  </si>
-  <si>
-    <t>6조 5629억 7412만</t>
-  </si>
-  <si>
-    <t>사나이기백황</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EC%82%AC%EB%82%98%EC%9D%B4%EA%B8%B0%EB%B0%B1%ED%99%A9</t>
-  </si>
-  <si>
-    <t>3조 8303억 3845만</t>
-  </si>
-  <si>
-    <t>토미오카상</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%ED%86%A0%EB%AF%B8%EC%98%A4%EC%B9%B4%EC%83%81</t>
-  </si>
-  <si>
-    <t>3조 3002억 4541만</t>
-  </si>
-  <si>
-    <t>평평이형</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%ED%8F%89%ED%8F%89%EC%9D%B4%ED%98%95</t>
-  </si>
-  <si>
-    <t>3조 906억 3513만</t>
-  </si>
-  <si>
-    <t>천칠</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EC%B2%9C%EC%B9%A0</t>
-  </si>
-  <si>
-    <t>팔라딘</t>
-  </si>
-  <si>
-    <t>2조 6702억 2482만</t>
-  </si>
-  <si>
-    <t>토니워터</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%ED%86%A0%EB%8B%88%EC%9B%8C%ED%84%B0</t>
-  </si>
-  <si>
-    <t>2조 6162억 1545만</t>
-  </si>
-  <si>
-    <t>펑풀</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%ED%8E%91%ED%92%80</t>
-  </si>
-  <si>
-    <t>2조 4885억 7115만</t>
-  </si>
-  <si>
-    <t>화살대</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%ED%99%94%EC%82%B4%EB%8C%80</t>
-  </si>
-  <si>
-    <t>2조 4258억 6186만</t>
-  </si>
-  <si>
-    <t>런닝래빗</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EB%9F%B0%EB%8B%9D%EB%9E%98%EB%B9%97</t>
-  </si>
-  <si>
-    <t>2조 4177억 8071만</t>
-  </si>
-  <si>
-    <t>피어난</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%ED%94%BC%EC%96%B4%EB%82%9C</t>
-  </si>
-  <si>
-    <t>2조 305억 8537만</t>
-  </si>
-  <si>
-    <t>샤스찌에</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EC%83%A4%EC%8A%A4%EC%B0%8C%EC%97%90</t>
-  </si>
-  <si>
-    <t>1조 4976억 9640만</t>
-  </si>
-  <si>
-    <t>보동핑</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EB%B3%B4%EB%8F%99%ED%95%91</t>
-  </si>
-  <si>
-    <t>1조 1820억 5434만</t>
-  </si>
-  <si>
-    <t>싸토루</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EC%8B%B8%ED%86%A0%EB%A3%A8</t>
-  </si>
-  <si>
-    <t>95</t>
-  </si>
-  <si>
-    <t>1조 1480억 9108만</t>
-  </si>
-  <si>
-    <t>지니좋아요</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EC%A7%80%EB%8B%88%EC%A2%8B%EC%95%84%EC%9A%94</t>
-  </si>
-  <si>
-    <t>1조 666억 9786만</t>
-  </si>
-  <si>
-    <t>2026년1월30일</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=2026%EB%85%841%EC%9B%9430%EC%9D%BC</t>
-  </si>
-  <si>
-    <t>1조 129억 4198만</t>
-  </si>
-  <si>
-    <t>찐곽정근</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EC%B0%90%EA%B3%BD%EC%A0%95%EA%B7%BC</t>
-  </si>
-  <si>
-    <t>1조 24억 1640만</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%ED%99%8D%EC%B6%98%EC%82%BC</t>
-  </si>
-  <si>
-    <t>8747억 2403만</t>
-  </si>
-  <si>
-    <t>Targa</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=Targa</t>
-  </si>
-  <si>
-    <t>94</t>
-  </si>
-  <si>
-    <t>5665억 5826만</t>
-  </si>
-  <si>
-    <t>애둘이에요</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EC%95%A0%EB%91%98%EC%9D%B4%EC%97%90%EC%9A%94</t>
-  </si>
-  <si>
-    <t>93</t>
-  </si>
-  <si>
-    <t>5424억 3794만</t>
-  </si>
-  <si>
-    <t>짱창훈</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EC%A7%B1%EC%B0%BD%ED%9B%88</t>
-  </si>
-  <si>
-    <t>3382억 604만</t>
-  </si>
-  <si>
     <t>구리구리뽕리</t>
   </si>
   <si>
@@ -1472,7 +1460,7 @@
     <t>https://mgf.gg/contents/character.php?n=%EB%AF%BC%ED%97%A4</t>
   </si>
   <si>
-    <t>12조 8020억 1758만</t>
+    <t>13조 4832억 9129만</t>
   </si>
   <si>
     <t>세계챔피언</t>
@@ -1490,7 +1478,16 @@
     <t>https://mgf.gg/contents/character.php?n=I%EB%9D%BC%ED%97%ACI</t>
   </si>
   <si>
-    <t>3조 3361억 4225만</t>
+    <t>3조 3854억 4624만</t>
+  </si>
+  <si>
+    <t>찐썽잉</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EC%B0%90%EC%8D%BD%EC%9E%89</t>
+  </si>
+  <si>
+    <t>2조 5906억 6272만</t>
   </si>
   <si>
     <t>건야웅</t>
@@ -1502,15 +1499,6 @@
     <t>2조 4543억 8797만</t>
   </si>
   <si>
-    <t>찐썽잉</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EC%B0%90%EC%8D%BD%EC%9E%89</t>
-  </si>
-  <si>
-    <t>2조 2859억 6115만</t>
-  </si>
-  <si>
     <t>보꿍</t>
   </si>
   <si>
@@ -1544,7 +1532,7 @@
     <t>https://mgf.gg/contents/character.php?n=%EB%A0%88%EC%A0%9C%EB%82%B4%EA%BA%BC%EC%95%BC</t>
   </si>
   <si>
-    <t>9440억 8488만</t>
+    <t>9811억 2977만</t>
   </si>
   <si>
     <t>묨밍</t>
@@ -1625,7 +1613,7 @@
     <t>https://mgf.gg/contents/character.php?n=%ED%98%BC%EC%9E%90%EA%B0%80%EC%B5%9C%EA%B3%A0</t>
   </si>
   <si>
-    <t>4366억 6830만</t>
+    <t>4484억 5846만</t>
   </si>
   <si>
     <t>깝용잉</t>
@@ -1643,7 +1631,7 @@
     <t>https://mgf.gg/contents/character.php?n=%EB%A7%9D%EB%B3%B5%EB%B3%B5</t>
   </si>
   <si>
-    <t>3876억 9482만</t>
+    <t>4161억 969만</t>
   </si>
   <si>
     <t>모몬쌍</t>
@@ -1652,7 +1640,7 @@
     <t>https://mgf.gg/contents/character.php?n=%EB%AA%A8%EB%AA%AC%EC%8C%8D</t>
   </si>
   <si>
-    <t>2497억 5284만</t>
+    <t>2679억 4512만</t>
   </si>
   <si>
     <t>우주강아지</t>
@@ -1673,7 +1661,16 @@
     <t>92</t>
   </si>
   <si>
-    <t>1787억 2037만</t>
+    <t>1801억 3527만</t>
+  </si>
+  <si>
+    <t>이진니</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EC%9D%B4%EC%A7%84%EB%8B%88</t>
+  </si>
+  <si>
+    <t>970억 5432만</t>
   </si>
   <si>
     <t>봉오리</t>
@@ -1685,16 +1682,7 @@
     <t>87</t>
   </si>
   <si>
-    <t>919억 4970만</t>
-  </si>
-  <si>
-    <t>이진니</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EC%9D%B4%EC%A7%84%EB%8B%88</t>
-  </si>
-  <si>
-    <t>902억 7225만</t>
+    <t>921억 1003만</t>
   </si>
   <si>
     <t>만년설딸기</t>
@@ -1703,10 +1691,10 @@
     <t>https://mgf.gg/contents/character.php?n=%EB%A7%8C%EB%85%84%EC%84%A4%EB%94%B8%EA%B8%B0</t>
   </si>
   <si>
-    <t>84</t>
-  </si>
-  <si>
-    <t>230억 2754만</t>
+    <t>85</t>
+  </si>
+  <si>
+    <t>248억 7797만</t>
   </si>
 </sst>
 </file>
@@ -2346,7 +2334,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J30"/>
+  <dimension ref="A1:J29"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -2446,10 +2434,10 @@
         <v>80</v>
       </c>
       <c r="H3" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="I3" s="2" t="s">
         <v>81</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>82</v>
       </c>
       <c r="J3" s="2" t="s">
         <v>24</v>
@@ -2460,28 +2448,28 @@
         <v>13</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="D4" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="E4" s="2" t="s">
+      <c r="F4" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="F4" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="G4" s="2" t="s">
+      <c r="H4" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="I4" s="2" t="s">
         <v>87</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>88</v>
       </c>
       <c r="J4" s="2" t="s">
         <v>24</v>
@@ -2492,28 +2480,28 @@
         <v>13</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="D5" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E5" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="D5" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="E5" s="2" t="s">
+      <c r="F5" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="G5" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="F5" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="G5" s="2" t="s">
+      <c r="H5" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="I5" s="2" t="s">
         <v>92</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>93</v>
       </c>
       <c r="J5" s="2" t="s">
         <v>24</v>
@@ -2524,25 +2512,25 @@
         <v>13</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="D6" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="E6" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="D6" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="E6" s="2" t="s">
+      <c r="F6" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="G6" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="F6" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="G6" s="2" t="s">
+      <c r="H6" s="2" t="s">
         <v>97</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>81</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>98</v>
@@ -2571,10 +2559,10 @@
         <v>79</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>81</v>
+        <v>97</v>
       </c>
       <c r="I7" s="2" t="s">
         <v>102</v>
@@ -2603,7 +2591,7 @@
         <v>79</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H8" s="2" t="s">
         <v>106</v>
@@ -2638,7 +2626,7 @@
         <v>111</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I9" s="2" t="s">
         <v>112</v>
@@ -2670,7 +2658,7 @@
         <v>73</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I10" s="2" t="s">
         <v>116</v>
@@ -2731,10 +2719,10 @@
         <v>79</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I12" s="2" t="s">
         <v>126</v>
@@ -2798,7 +2786,7 @@
         <v>73</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I14" s="2" t="s">
         <v>134</v>
@@ -2894,10 +2882,10 @@
         <v>111</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="J17" s="2" t="s">
         <v>24</v>
@@ -2908,16 +2896,16 @@
         <v>13</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F18" s="2" t="s">
         <v>79</v>
@@ -2929,7 +2917,7 @@
         <v>121</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="J18" s="2" t="s">
         <v>24</v>
@@ -2940,25 +2928,25 @@
         <v>13</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>79</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>73</v>
+        <v>111</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>155</v>
+        <v>86</v>
       </c>
       <c r="I19" s="2" t="s">
         <v>156</v>
@@ -2987,10 +2975,10 @@
         <v>79</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>111</v>
+        <v>73</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>87</v>
+        <v>142</v>
       </c>
       <c r="I20" s="2" t="s">
         <v>160</v>
@@ -3022,7 +3010,7 @@
         <v>73</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>155</v>
+        <v>142</v>
       </c>
       <c r="I21" s="2" t="s">
         <v>164</v>
@@ -3054,7 +3042,7 @@
         <v>111</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>155</v>
+        <v>142</v>
       </c>
       <c r="I22" s="2" t="s">
         <v>168</v>
@@ -3086,7 +3074,7 @@
         <v>73</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I23" s="2" t="s">
         <v>172</v>
@@ -3118,7 +3106,7 @@
         <v>80</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="I24" s="2" t="s">
         <v>176</v>
@@ -3150,7 +3138,7 @@
         <v>180</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="I25" s="2" t="s">
         <v>181</v>
@@ -3179,10 +3167,10 @@
         <v>79</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>142</v>
+        <v>86</v>
       </c>
       <c r="I26" s="2" t="s">
         <v>185</v>
@@ -3211,10 +3199,10 @@
         <v>79</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>97</v>
+        <v>73</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>121</v>
+        <v>147</v>
       </c>
       <c r="I27" s="2" t="s">
         <v>189</v>
@@ -3243,10 +3231,10 @@
         <v>79</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>87</v>
+        <v>121</v>
       </c>
       <c r="I28" s="2" t="s">
         <v>193</v>
@@ -3287,40 +3275,8 @@
         <v>24</v>
       </c>
     </row>
-    <row r="30" spans="1:10">
-      <c r="A30" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="E30" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="F30" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="G30" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="H30" s="2" t="s">
-        <v>202</v>
-      </c>
-      <c r="I30" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="J30" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:J30"/>
+  <autoFilter ref="A1:J29"/>
   <hyperlinks>
     <hyperlink ref="E2" r:id="rId1"/>
     <hyperlink ref="E3" r:id="rId2"/>
@@ -3350,7 +3306,6 @@
     <hyperlink ref="E27" r:id="rId26"/>
     <hyperlink ref="E28" r:id="rId27"/>
     <hyperlink ref="E29" r:id="rId28"/>
-    <hyperlink ref="E30" r:id="rId29"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3411,13 +3366,13 @@
         <v>70</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>79</v>
@@ -3429,7 +3384,7 @@
         <v>106</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="J2" s="2" t="s">
         <v>34</v>
@@ -3443,25 +3398,25 @@
         <v>76</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>79</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H3" s="2" t="s">
         <v>106</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="J3" s="2" t="s">
         <v>34</v>
@@ -3472,16 +3427,16 @@
         <v>25</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>79</v>
@@ -3493,7 +3448,7 @@
         <v>106</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="J4" s="2" t="s">
         <v>34</v>
@@ -3504,16 +3459,16 @@
         <v>25</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>79</v>
@@ -3525,7 +3480,7 @@
         <v>106</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="J5" s="2" t="s">
         <v>34</v>
@@ -3536,16 +3491,16 @@
         <v>25</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>79</v>
@@ -3554,10 +3509,10 @@
         <v>111</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="J6" s="2" t="s">
         <v>34</v>
@@ -3571,13 +3526,13 @@
         <v>99</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>79</v>
@@ -3586,10 +3541,10 @@
         <v>73</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="J7" s="2" t="s">
         <v>34</v>
@@ -3603,13 +3558,13 @@
         <v>103</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>79</v>
@@ -3618,10 +3573,10 @@
         <v>73</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="J8" s="2" t="s">
         <v>34</v>
@@ -3635,13 +3590,13 @@
         <v>108</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>79</v>
@@ -3650,10 +3605,10 @@
         <v>111</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="J9" s="2" t="s">
         <v>34</v>
@@ -3667,25 +3622,25 @@
         <v>113</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>79</v>
       </c>
       <c r="G10" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="H10" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="H10" s="2" t="s">
-        <v>87</v>
-      </c>
       <c r="I10" s="2" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
       <c r="J10" s="2" t="s">
         <v>34</v>
@@ -3699,25 +3654,25 @@
         <v>117</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>79</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H11" s="2" t="s">
         <v>121</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="J11" s="2" t="s">
         <v>34</v>
@@ -3731,13 +3686,13 @@
         <v>123</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>234</v>
+        <v>229</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>234</v>
+        <v>229</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>79</v>
@@ -3746,10 +3701,10 @@
         <v>80</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="J12" s="2" t="s">
         <v>34</v>
@@ -3763,13 +3718,13 @@
         <v>127</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>79</v>
@@ -3778,10 +3733,10 @@
         <v>73</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="J13" s="2" t="s">
         <v>34</v>
@@ -3795,25 +3750,25 @@
         <v>131</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>79</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="H14" s="2" t="s">
         <v>121</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="J14" s="2" t="s">
         <v>34</v>
@@ -3827,13 +3782,13 @@
         <v>135</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="F15" s="2" t="s">
         <v>79</v>
@@ -3842,10 +3797,10 @@
         <v>73</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="J15" s="2" t="s">
         <v>34</v>
@@ -3859,13 +3814,13 @@
         <v>139</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>79</v>
@@ -3874,10 +3829,10 @@
         <v>80</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="J16" s="2" t="s">
         <v>34</v>
@@ -3891,25 +3846,25 @@
         <v>144</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="F17" s="2" t="s">
         <v>79</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>155</v>
+        <v>142</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
       <c r="J17" s="2" t="s">
         <v>34</v>
@@ -3920,16 +3875,16 @@
         <v>25</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="F18" s="2" t="s">
         <v>79</v>
@@ -3941,7 +3896,7 @@
         <v>197</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="J18" s="2" t="s">
         <v>34</v>
@@ -3952,28 +3907,28 @@
         <v>25</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>79</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>155</v>
+        <v>142</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="J19" s="2" t="s">
         <v>34</v>
@@ -3987,13 +3942,13 @@
         <v>157</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="F20" s="2" t="s">
         <v>79</v>
@@ -4005,7 +3960,7 @@
         <v>197</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="J20" s="2" t="s">
         <v>34</v>
@@ -4019,25 +3974,25 @@
         <v>161</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="F21" s="2" t="s">
         <v>79</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H21" s="2" t="s">
         <v>197</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="J21" s="2" t="s">
         <v>34</v>
@@ -4051,25 +4006,25 @@
         <v>165</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="F22" s="2" t="s">
         <v>79</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="J22" s="2" t="s">
         <v>34</v>
@@ -4083,13 +4038,13 @@
         <v>169</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="F23" s="2" t="s">
         <v>79</v>
@@ -4101,7 +4056,7 @@
         <v>197</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>271</v>
+        <v>266</v>
       </c>
       <c r="J23" s="2" t="s">
         <v>34</v>
@@ -4115,13 +4070,13 @@
         <v>173</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="F24" s="2" t="s">
         <v>79</v>
@@ -4133,7 +4088,7 @@
         <v>197</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>274</v>
+        <v>269</v>
       </c>
       <c r="J24" s="2" t="s">
         <v>34</v>
@@ -4147,25 +4102,25 @@
         <v>177</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
       <c r="F25" s="2" t="s">
         <v>79</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
       <c r="J25" s="2" t="s">
         <v>34</v>
@@ -4185,7 +4140,7 @@
         <v>33</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>278</v>
+        <v>273</v>
       </c>
       <c r="F26" s="2" t="s">
         <v>72</v>
@@ -4194,10 +4149,10 @@
         <v>120</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>279</v>
+        <v>274</v>
       </c>
       <c r="J26" s="2" t="s">
         <v>34</v>
@@ -4211,13 +4166,13 @@
         <v>186</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>281</v>
+        <v>276</v>
       </c>
       <c r="F27" s="2" t="s">
         <v>79</v>
@@ -4226,10 +4181,10 @@
         <v>73</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
       <c r="J27" s="2" t="s">
         <v>34</v>
@@ -4243,13 +4198,13 @@
         <v>190</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
       <c r="F28" s="2" t="s">
         <v>79</v>
@@ -4258,10 +4213,10 @@
         <v>80</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="J28" s="2" t="s">
         <v>34</v>
@@ -4275,13 +4230,13 @@
         <v>194</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>289</v>
+        <v>284</v>
       </c>
       <c r="F29" s="2" t="s">
         <v>79</v>
@@ -4290,10 +4245,10 @@
         <v>111</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
       <c r="I29" s="2" t="s">
-        <v>290</v>
+        <v>285</v>
       </c>
       <c r="J29" s="2" t="s">
         <v>34</v>
@@ -4304,28 +4259,28 @@
         <v>25</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>199</v>
+        <v>286</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="F30" s="2" t="s">
         <v>79</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>294</v>
+        <v>290</v>
       </c>
       <c r="J30" s="2" t="s">
         <v>34</v>
@@ -4423,25 +4378,25 @@
         <v>70</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>79</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>106</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="J2" s="2" t="s">
         <v>34</v>
@@ -4455,13 +4410,13 @@
         <v>76</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>79</v>
@@ -4470,10 +4425,10 @@
         <v>80</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>81</v>
+        <v>97</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="J3" s="2" t="s">
         <v>34</v>
@@ -4484,16 +4439,16 @@
         <v>35</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>302</v>
+        <v>298</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>79</v>
@@ -4505,7 +4460,7 @@
         <v>106</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>303</v>
+        <v>299</v>
       </c>
       <c r="J4" s="2" t="s">
         <v>34</v>
@@ -4516,16 +4471,16 @@
         <v>35</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>79</v>
@@ -4537,7 +4492,7 @@
         <v>106</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>306</v>
+        <v>302</v>
       </c>
       <c r="J5" s="2" t="s">
         <v>34</v>
@@ -4548,16 +4503,16 @@
         <v>35</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>307</v>
+        <v>303</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>307</v>
+        <v>303</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>79</v>
@@ -4569,7 +4524,7 @@
         <v>106</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>309</v>
+        <v>305</v>
       </c>
       <c r="J6" s="2" t="s">
         <v>34</v>
@@ -4583,13 +4538,13 @@
         <v>99</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>310</v>
+        <v>306</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>310</v>
+        <v>306</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>79</v>
@@ -4601,7 +4556,7 @@
         <v>106</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="J7" s="2" t="s">
         <v>34</v>
@@ -4615,25 +4570,25 @@
         <v>103</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>79</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="H8" s="2" t="s">
         <v>106</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="J8" s="2" t="s">
         <v>34</v>
@@ -4647,25 +4602,25 @@
         <v>108</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>79</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H9" s="2" t="s">
         <v>121</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="J9" s="2" t="s">
         <v>34</v>
@@ -4679,13 +4634,13 @@
         <v>113</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>79</v>
@@ -4697,7 +4652,7 @@
         <v>121</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="J10" s="2" t="s">
         <v>34</v>
@@ -4711,13 +4666,13 @@
         <v>117</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>79</v>
@@ -4729,7 +4684,7 @@
         <v>121</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="J11" s="2" t="s">
         <v>34</v>
@@ -4743,25 +4698,25 @@
         <v>123</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>79</v>
       </c>
       <c r="G12" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="H12" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="H12" s="2" t="s">
-        <v>87</v>
-      </c>
       <c r="I12" s="2" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="J12" s="2" t="s">
         <v>34</v>
@@ -4775,13 +4730,13 @@
         <v>127</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>79</v>
@@ -4790,10 +4745,10 @@
         <v>73</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>155</v>
+        <v>142</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="J13" s="2" t="s">
         <v>34</v>
@@ -4813,19 +4768,19 @@
         <v>42</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>72</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="J14" s="2" t="s">
         <v>34</v>
@@ -4839,13 +4794,13 @@
         <v>135</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>334</v>
+        <v>330</v>
       </c>
       <c r="F15" s="2" t="s">
         <v>79</v>
@@ -4857,7 +4812,7 @@
         <v>121</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>335</v>
+        <v>331</v>
       </c>
       <c r="J15" s="2" t="s">
         <v>34</v>
@@ -4871,25 +4826,25 @@
         <v>139</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>336</v>
+        <v>332</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>336</v>
+        <v>332</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>337</v>
+        <v>333</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>79</v>
       </c>
       <c r="G16" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="H16" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="H16" s="2" t="s">
-        <v>87</v>
-      </c>
       <c r="I16" s="2" t="s">
-        <v>338</v>
+        <v>334</v>
       </c>
       <c r="J16" s="2" t="s">
         <v>34</v>
@@ -4903,13 +4858,13 @@
         <v>144</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>339</v>
+        <v>335</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>339</v>
+        <v>335</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>340</v>
+        <v>336</v>
       </c>
       <c r="F17" s="2" t="s">
         <v>79</v>
@@ -4921,7 +4876,7 @@
         <v>197</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>341</v>
+        <v>337</v>
       </c>
       <c r="J17" s="2" t="s">
         <v>34</v>
@@ -4932,16 +4887,16 @@
         <v>35</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>342</v>
+        <v>338</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>342</v>
+        <v>338</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>343</v>
+        <v>339</v>
       </c>
       <c r="F18" s="2" t="s">
         <v>79</v>
@@ -4950,10 +4905,10 @@
         <v>111</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>344</v>
+        <v>340</v>
       </c>
       <c r="J18" s="2" t="s">
         <v>34</v>
@@ -4964,16 +4919,16 @@
         <v>35</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>345</v>
+        <v>341</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>345</v>
+        <v>341</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>346</v>
+        <v>342</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>79</v>
@@ -4985,7 +4940,7 @@
         <v>197</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>347</v>
+        <v>343</v>
       </c>
       <c r="J19" s="2" t="s">
         <v>34</v>
@@ -4999,13 +4954,13 @@
         <v>157</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>348</v>
+        <v>344</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>348</v>
+        <v>344</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>349</v>
+        <v>345</v>
       </c>
       <c r="F20" s="2" t="s">
         <v>79</v>
@@ -5017,7 +4972,7 @@
         <v>197</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="J20" s="2" t="s">
         <v>34</v>
@@ -5031,13 +4986,13 @@
         <v>161</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>351</v>
+        <v>347</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>351</v>
+        <v>347</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>352</v>
+        <v>348</v>
       </c>
       <c r="F21" s="2" t="s">
         <v>79</v>
@@ -5049,7 +5004,7 @@
         <v>197</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>353</v>
+        <v>349</v>
       </c>
       <c r="J21" s="2" t="s">
         <v>34</v>
@@ -5063,13 +5018,13 @@
         <v>165</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>354</v>
+        <v>350</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>354</v>
+        <v>350</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>355</v>
+        <v>351</v>
       </c>
       <c r="F22" s="2" t="s">
         <v>79</v>
@@ -5078,10 +5033,10 @@
         <v>80</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>356</v>
+        <v>352</v>
       </c>
       <c r="J22" s="2" t="s">
         <v>34</v>
@@ -5095,25 +5050,25 @@
         <v>169</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>357</v>
+        <v>353</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>357</v>
+        <v>353</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>358</v>
+        <v>354</v>
       </c>
       <c r="F23" s="2" t="s">
         <v>79</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>359</v>
+        <v>355</v>
       </c>
       <c r="J23" s="2" t="s">
         <v>34</v>
@@ -5127,13 +5082,13 @@
         <v>173</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>360</v>
+        <v>356</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>360</v>
+        <v>356</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>361</v>
+        <v>357</v>
       </c>
       <c r="F24" s="2" t="s">
         <v>79</v>
@@ -5142,10 +5097,10 @@
         <v>111</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>362</v>
+        <v>358</v>
       </c>
       <c r="J24" s="2" t="s">
         <v>34</v>
@@ -5159,13 +5114,13 @@
         <v>177</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>363</v>
+        <v>359</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>363</v>
+        <v>359</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>364</v>
+        <v>360</v>
       </c>
       <c r="F25" s="2" t="s">
         <v>79</v>
@@ -5174,10 +5129,10 @@
         <v>73</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>365</v>
+        <v>361</v>
       </c>
       <c r="J25" s="2" t="s">
         <v>34</v>
@@ -5191,13 +5146,13 @@
         <v>182</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>366</v>
+        <v>362</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>366</v>
+        <v>362</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="F26" s="2" t="s">
         <v>79</v>
@@ -5206,10 +5161,10 @@
         <v>73</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>368</v>
+        <v>364</v>
       </c>
       <c r="J26" s="2" t="s">
         <v>34</v>
@@ -5223,13 +5178,13 @@
         <v>186</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>369</v>
+        <v>365</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>369</v>
+        <v>365</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="F27" s="2" t="s">
         <v>79</v>
@@ -5238,10 +5193,10 @@
         <v>111</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>371</v>
+        <v>367</v>
       </c>
       <c r="J27" s="2" t="s">
         <v>34</v>
@@ -5255,13 +5210,13 @@
         <v>190</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>372</v>
+        <v>368</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>372</v>
+        <v>368</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>373</v>
+        <v>369</v>
       </c>
       <c r="F28" s="2" t="s">
         <v>79</v>
@@ -5270,10 +5225,10 @@
         <v>73</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>374</v>
+        <v>370</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>375</v>
+        <v>371</v>
       </c>
       <c r="J28" s="2" t="s">
         <v>34</v>
@@ -5287,25 +5242,25 @@
         <v>194</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>376</v>
+        <v>372</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>376</v>
+        <v>372</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="F29" s="2" t="s">
         <v>79</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>378</v>
+        <v>374</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>374</v>
+        <v>370</v>
       </c>
       <c r="I29" s="2" t="s">
-        <v>379</v>
+        <v>375</v>
       </c>
       <c r="J29" s="2" t="s">
         <v>34</v>
@@ -5316,28 +5271,28 @@
         <v>35</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>199</v>
+        <v>286</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>380</v>
+        <v>376</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>380</v>
+        <v>376</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>381</v>
+        <v>377</v>
       </c>
       <c r="F30" s="2" t="s">
         <v>79</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>374</v>
+        <v>370</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>382</v>
+        <v>378</v>
       </c>
       <c r="J30" s="2" t="s">
         <v>34</v>
@@ -5435,25 +5390,25 @@
         <v>70</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>383</v>
+        <v>379</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>383</v>
+        <v>379</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>384</v>
+        <v>380</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>79</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>74</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>385</v>
+        <v>381</v>
       </c>
       <c r="J2" s="2" t="s">
         <v>34</v>
@@ -5467,13 +5422,13 @@
         <v>76</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>386</v>
+        <v>382</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>386</v>
+        <v>382</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>387</v>
+        <v>383</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>79</v>
@@ -5482,10 +5437,10 @@
         <v>73</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>81</v>
+        <v>97</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>388</v>
+        <v>384</v>
       </c>
       <c r="J3" s="2" t="s">
         <v>34</v>
@@ -5496,28 +5451,28 @@
         <v>43</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>389</v>
+        <v>385</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>389</v>
+        <v>385</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>390</v>
+        <v>386</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>79</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>378</v>
+        <v>374</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>81</v>
+        <v>97</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>391</v>
+        <v>387</v>
       </c>
       <c r="J4" s="2" t="s">
         <v>34</v>
@@ -5528,28 +5483,28 @@
         <v>43</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>392</v>
+        <v>388</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>392</v>
+        <v>388</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>393</v>
+        <v>389</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>79</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="H5" s="2" t="s">
         <v>121</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
       <c r="J5" s="2" t="s">
         <v>34</v>
@@ -5560,28 +5515,28 @@
         <v>43</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>395</v>
+        <v>391</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>395</v>
+        <v>391</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>396</v>
+        <v>392</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>79</v>
       </c>
       <c r="G6" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="H6" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="H6" s="2" t="s">
-        <v>87</v>
-      </c>
       <c r="I6" s="2" t="s">
-        <v>397</v>
+        <v>393</v>
       </c>
       <c r="J6" s="2" t="s">
         <v>34</v>
@@ -5595,25 +5550,25 @@
         <v>99</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>398</v>
+        <v>394</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>398</v>
+        <v>394</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>399</v>
+        <v>395</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>79</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>378</v>
+        <v>374</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>400</v>
+        <v>396</v>
       </c>
       <c r="J7" s="2" t="s">
         <v>34</v>
@@ -5633,7 +5588,7 @@
         <v>52</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>401</v>
+        <v>397</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>72</v>
@@ -5642,10 +5597,10 @@
         <v>73</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>402</v>
+        <v>398</v>
       </c>
       <c r="J8" s="2" t="s">
         <v>34</v>
@@ -5659,25 +5614,25 @@
         <v>108</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>403</v>
+        <v>399</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>403</v>
+        <v>399</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>404</v>
+        <v>400</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>79</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>378</v>
+        <v>374</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>405</v>
+        <v>401</v>
       </c>
       <c r="J9" s="2" t="s">
         <v>34</v>
@@ -5691,13 +5646,13 @@
         <v>113</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>406</v>
+        <v>402</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>406</v>
+        <v>402</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>407</v>
+        <v>403</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>79</v>
@@ -5709,7 +5664,7 @@
         <v>121</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>408</v>
+        <v>404</v>
       </c>
       <c r="J10" s="2" t="s">
         <v>34</v>
@@ -5723,13 +5678,13 @@
         <v>117</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>409</v>
+        <v>405</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>409</v>
+        <v>405</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>410</v>
+        <v>406</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>79</v>
@@ -5738,10 +5693,10 @@
         <v>111</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>411</v>
+        <v>407</v>
       </c>
       <c r="J11" s="2" t="s">
         <v>34</v>
@@ -5755,13 +5710,13 @@
         <v>123</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>412</v>
+        <v>408</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>412</v>
+        <v>408</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>413</v>
+        <v>409</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>79</v>
@@ -5773,7 +5728,7 @@
         <v>197</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>414</v>
+        <v>410</v>
       </c>
       <c r="J12" s="2" t="s">
         <v>34</v>
@@ -5787,13 +5742,13 @@
         <v>127</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>415</v>
+        <v>411</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>415</v>
+        <v>411</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>416</v>
+        <v>412</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>79</v>
@@ -5805,7 +5760,7 @@
         <v>197</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>417</v>
+        <v>413</v>
       </c>
       <c r="J13" s="2" t="s">
         <v>34</v>
@@ -5819,13 +5774,13 @@
         <v>131</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>418</v>
+        <v>414</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>418</v>
+        <v>414</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>419</v>
+        <v>415</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>79</v>
@@ -5837,7 +5792,7 @@
         <v>197</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>420</v>
+        <v>416</v>
       </c>
       <c r="J14" s="2" t="s">
         <v>34</v>
@@ -5851,13 +5806,13 @@
         <v>135</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>421</v>
+        <v>417</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>421</v>
+        <v>417</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>422</v>
+        <v>418</v>
       </c>
       <c r="F15" s="2" t="s">
         <v>79</v>
@@ -5869,7 +5824,7 @@
         <v>197</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>423</v>
+        <v>419</v>
       </c>
       <c r="J15" s="2" t="s">
         <v>34</v>
@@ -5883,13 +5838,13 @@
         <v>139</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>424</v>
+        <v>420</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>424</v>
+        <v>420</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>425</v>
+        <v>421</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>79</v>
@@ -5901,7 +5856,7 @@
         <v>197</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>426</v>
+        <v>422</v>
       </c>
       <c r="J16" s="2" t="s">
         <v>34</v>
@@ -5915,13 +5870,13 @@
         <v>144</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>427</v>
+        <v>423</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>427</v>
+        <v>423</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>428</v>
+        <v>424</v>
       </c>
       <c r="F17" s="2" t="s">
         <v>79</v>
@@ -5933,7 +5888,7 @@
         <v>197</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>429</v>
+        <v>425</v>
       </c>
       <c r="J17" s="2" t="s">
         <v>34</v>
@@ -5944,16 +5899,16 @@
         <v>43</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>430</v>
+        <v>426</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>430</v>
+        <v>426</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>431</v>
+        <v>427</v>
       </c>
       <c r="F18" s="2" t="s">
         <v>79</v>
@@ -5965,7 +5920,7 @@
         <v>197</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>432</v>
+        <v>428</v>
       </c>
       <c r="J18" s="2" t="s">
         <v>34</v>
@@ -5976,16 +5931,16 @@
         <v>43</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>433</v>
+        <v>429</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>433</v>
+        <v>429</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>434</v>
+        <v>430</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>79</v>
@@ -5994,10 +5949,10 @@
         <v>80</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>435</v>
+        <v>431</v>
       </c>
       <c r="J19" s="2" t="s">
         <v>34</v>
@@ -6011,13 +5966,13 @@
         <v>157</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>436</v>
+        <v>432</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>436</v>
+        <v>432</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>437</v>
+        <v>433</v>
       </c>
       <c r="F20" s="2" t="s">
         <v>79</v>
@@ -6029,7 +5984,7 @@
         <v>197</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>438</v>
+        <v>434</v>
       </c>
       <c r="J20" s="2" t="s">
         <v>34</v>
@@ -6043,13 +5998,13 @@
         <v>161</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>439</v>
+        <v>435</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>439</v>
+        <v>435</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>440</v>
+        <v>436</v>
       </c>
       <c r="F21" s="2" t="s">
         <v>79</v>
@@ -6061,7 +6016,7 @@
         <v>197</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>441</v>
+        <v>437</v>
       </c>
       <c r="J21" s="2" t="s">
         <v>34</v>
@@ -6075,13 +6030,13 @@
         <v>165</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>442</v>
+        <v>438</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>442</v>
+        <v>438</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>443</v>
+        <v>439</v>
       </c>
       <c r="F22" s="2" t="s">
         <v>79</v>
@@ -6090,10 +6045,10 @@
         <v>73</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>444</v>
+        <v>440</v>
       </c>
       <c r="J22" s="2" t="s">
         <v>34</v>
@@ -6107,13 +6062,13 @@
         <v>169</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>445</v>
+        <v>441</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>445</v>
+        <v>441</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>446</v>
+        <v>442</v>
       </c>
       <c r="F23" s="2" t="s">
         <v>79</v>
@@ -6122,10 +6077,10 @@
         <v>111</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>447</v>
+        <v>443</v>
       </c>
       <c r="J23" s="2" t="s">
         <v>34</v>
@@ -6139,13 +6094,13 @@
         <v>173</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>448</v>
+        <v>444</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>448</v>
+        <v>444</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>449</v>
+        <v>445</v>
       </c>
       <c r="F24" s="2" t="s">
         <v>79</v>
@@ -6154,10 +6109,10 @@
         <v>111</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>450</v>
+        <v>446</v>
       </c>
       <c r="J24" s="2" t="s">
         <v>34</v>
@@ -6171,13 +6126,13 @@
         <v>177</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>451</v>
+        <v>447</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>451</v>
+        <v>447</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>452</v>
+        <v>448</v>
       </c>
       <c r="F25" s="2" t="s">
         <v>79</v>
@@ -6189,7 +6144,7 @@
         <v>197</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>453</v>
+        <v>449</v>
       </c>
       <c r="J25" s="2" t="s">
         <v>34</v>
@@ -6203,13 +6158,13 @@
         <v>182</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>454</v>
+        <v>450</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>454</v>
+        <v>450</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>455</v>
+        <v>451</v>
       </c>
       <c r="F26" s="2" t="s">
         <v>79</v>
@@ -6218,10 +6173,10 @@
         <v>111</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>456</v>
+        <v>452</v>
       </c>
       <c r="J26" s="2" t="s">
         <v>34</v>
@@ -6235,13 +6190,13 @@
         <v>186</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>457</v>
+        <v>453</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>457</v>
+        <v>453</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>458</v>
+        <v>454</v>
       </c>
       <c r="F27" s="2" t="s">
         <v>79</v>
@@ -6250,10 +6205,10 @@
         <v>73</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>459</v>
+        <v>455</v>
       </c>
       <c r="J27" s="2" t="s">
         <v>34</v>
@@ -6267,13 +6222,13 @@
         <v>190</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>460</v>
+        <v>456</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>460</v>
+        <v>456</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>461</v>
+        <v>457</v>
       </c>
       <c r="F28" s="2" t="s">
         <v>79</v>
@@ -6282,10 +6237,10 @@
         <v>111</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>462</v>
+        <v>458</v>
       </c>
       <c r="J28" s="2" t="s">
         <v>34</v>
@@ -6299,25 +6254,25 @@
         <v>194</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>463</v>
+        <v>459</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>463</v>
+        <v>459</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>464</v>
+        <v>460</v>
       </c>
       <c r="F29" s="2" t="s">
         <v>79</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="I29" s="2" t="s">
-        <v>465</v>
+        <v>461</v>
       </c>
       <c r="J29" s="2" t="s">
         <v>34</v>
@@ -6328,28 +6283,28 @@
         <v>43</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>199</v>
+        <v>286</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>466</v>
+        <v>462</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>466</v>
+        <v>462</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>467</v>
+        <v>463</v>
       </c>
       <c r="F30" s="2" t="s">
         <v>79</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>378</v>
+        <v>374</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>468</v>
+        <v>464</v>
       </c>
       <c r="J30" s="2" t="s">
         <v>34</v>
@@ -6360,16 +6315,16 @@
         <v>43</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>469</v>
+        <v>465</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>470</v>
+        <v>466</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>470</v>
+        <v>466</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>471</v>
+        <v>467</v>
       </c>
       <c r="F31" s="2" t="s">
         <v>79</v>
@@ -6378,10 +6333,10 @@
         <v>73</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>472</v>
+        <v>468</v>
       </c>
       <c r="J31" s="2" t="s">
         <v>34</v>
@@ -6480,13 +6435,13 @@
         <v>70</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>473</v>
+        <v>469</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>473</v>
+        <v>469</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>474</v>
+        <v>470</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>79</v>
@@ -6495,10 +6450,10 @@
         <v>73</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>475</v>
+        <v>471</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>476</v>
+        <v>472</v>
       </c>
       <c r="J2" s="2" t="s">
         <v>34</v>
@@ -6518,7 +6473,7 @@
         <v>61</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>477</v>
+        <v>473</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>72</v>
@@ -6530,7 +6485,7 @@
         <v>74</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>478</v>
+        <v>474</v>
       </c>
       <c r="J3" s="2" t="s">
         <v>34</v>
@@ -6541,16 +6496,16 @@
         <v>53</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>479</v>
+        <v>475</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>479</v>
+        <v>475</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>480</v>
+        <v>476</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>79</v>
@@ -6562,7 +6517,7 @@
         <v>106</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>481</v>
+        <v>477</v>
       </c>
       <c r="J4" s="2" t="s">
         <v>34</v>
@@ -6573,16 +6528,16 @@
         <v>53</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>482</v>
+        <v>478</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>482</v>
+        <v>478</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>483</v>
+        <v>479</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>79</v>
@@ -6594,7 +6549,7 @@
         <v>106</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>484</v>
+        <v>480</v>
       </c>
       <c r="J5" s="2" t="s">
         <v>34</v>
@@ -6605,16 +6560,16 @@
         <v>53</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>485</v>
+        <v>481</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>485</v>
+        <v>481</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>486</v>
+        <v>482</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>79</v>
@@ -6626,7 +6581,7 @@
         <v>121</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>487</v>
+        <v>483</v>
       </c>
       <c r="J6" s="2" t="s">
         <v>34</v>
@@ -6640,25 +6595,25 @@
         <v>99</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>488</v>
+        <v>484</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>488</v>
+        <v>484</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>489</v>
+        <v>485</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>79</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>378</v>
+        <v>237</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>155</v>
+        <v>142</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>490</v>
+        <v>486</v>
       </c>
       <c r="J7" s="2" t="s">
         <v>34</v>
@@ -6672,25 +6627,25 @@
         <v>103</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>491</v>
+        <v>487</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>491</v>
+        <v>487</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>492</v>
+        <v>488</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>79</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>242</v>
+        <v>374</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>155</v>
+        <v>142</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>493</v>
+        <v>489</v>
       </c>
       <c r="J8" s="2" t="s">
         <v>34</v>
@@ -6704,13 +6659,13 @@
         <v>108</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>494</v>
+        <v>490</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>494</v>
+        <v>490</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>495</v>
+        <v>491</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>79</v>
@@ -6719,10 +6674,10 @@
         <v>73</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>155</v>
+        <v>142</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>496</v>
+        <v>492</v>
       </c>
       <c r="J9" s="2" t="s">
         <v>34</v>
@@ -6736,13 +6691,13 @@
         <v>113</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>497</v>
+        <v>493</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>497</v>
+        <v>493</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>498</v>
+        <v>494</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>79</v>
@@ -6751,10 +6706,10 @@
         <v>120</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>499</v>
+        <v>495</v>
       </c>
       <c r="J10" s="2" t="s">
         <v>34</v>
@@ -6768,13 +6723,13 @@
         <v>117</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>500</v>
+        <v>496</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>500</v>
+        <v>496</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>501</v>
+        <v>497</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>79</v>
@@ -6783,10 +6738,10 @@
         <v>73</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>502</v>
+        <v>498</v>
       </c>
       <c r="J11" s="2" t="s">
         <v>34</v>
@@ -6800,13 +6755,13 @@
         <v>123</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>503</v>
+        <v>499</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>503</v>
+        <v>499</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>504</v>
+        <v>500</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>79</v>
@@ -6815,10 +6770,10 @@
         <v>111</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>505</v>
+        <v>501</v>
       </c>
       <c r="J12" s="2" t="s">
         <v>34</v>
@@ -6832,13 +6787,13 @@
         <v>127</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>506</v>
+        <v>502</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>506</v>
+        <v>502</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>507</v>
+        <v>503</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>79</v>
@@ -6850,7 +6805,7 @@
         <v>197</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>508</v>
+        <v>504</v>
       </c>
       <c r="J13" s="2" t="s">
         <v>34</v>
@@ -6864,13 +6819,13 @@
         <v>131</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>509</v>
+        <v>505</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>509</v>
+        <v>505</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>510</v>
+        <v>506</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>79</v>
@@ -6882,7 +6837,7 @@
         <v>197</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>511</v>
+        <v>507</v>
       </c>
       <c r="J14" s="2" t="s">
         <v>34</v>
@@ -6896,25 +6851,25 @@
         <v>135</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>512</v>
+        <v>508</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>512</v>
+        <v>508</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>513</v>
+        <v>509</v>
       </c>
       <c r="F15" s="2" t="s">
         <v>79</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>514</v>
+        <v>510</v>
       </c>
       <c r="J15" s="2" t="s">
         <v>34</v>
@@ -6928,13 +6883,13 @@
         <v>139</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>515</v>
+        <v>511</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>515</v>
+        <v>511</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>516</v>
+        <v>512</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>79</v>
@@ -6946,7 +6901,7 @@
         <v>197</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>517</v>
+        <v>513</v>
       </c>
       <c r="J16" s="2" t="s">
         <v>34</v>
@@ -6960,13 +6915,13 @@
         <v>144</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>518</v>
+        <v>514</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>518</v>
+        <v>514</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>519</v>
+        <v>515</v>
       </c>
       <c r="F17" s="2" t="s">
         <v>79</v>
@@ -6975,10 +6930,10 @@
         <v>80</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>520</v>
+        <v>516</v>
       </c>
       <c r="J17" s="2" t="s">
         <v>34</v>
@@ -6989,16 +6944,16 @@
         <v>53</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>521</v>
+        <v>517</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>521</v>
+        <v>517</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>522</v>
+        <v>518</v>
       </c>
       <c r="F18" s="2" t="s">
         <v>79</v>
@@ -7007,10 +6962,10 @@
         <v>73</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>523</v>
+        <v>519</v>
       </c>
       <c r="J18" s="2" t="s">
         <v>34</v>
@@ -7021,28 +6976,28 @@
         <v>53</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>524</v>
+        <v>520</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>524</v>
+        <v>520</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>525</v>
+        <v>521</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>79</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>378</v>
+        <v>374</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="J19" s="2" t="s">
         <v>34</v>
@@ -7056,25 +7011,25 @@
         <v>157</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>527</v>
+        <v>523</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>527</v>
+        <v>523</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>528</v>
+        <v>524</v>
       </c>
       <c r="F20" s="2" t="s">
         <v>79</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>529</v>
+        <v>525</v>
       </c>
       <c r="J20" s="2" t="s">
         <v>34</v>
@@ -7088,25 +7043,25 @@
         <v>161</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>530</v>
+        <v>526</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>530</v>
+        <v>526</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>531</v>
+        <v>527</v>
       </c>
       <c r="F21" s="2" t="s">
         <v>79</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>532</v>
+        <v>528</v>
       </c>
       <c r="J21" s="2" t="s">
         <v>34</v>
@@ -7120,13 +7075,13 @@
         <v>165</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>533</v>
+        <v>529</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>533</v>
+        <v>529</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>534</v>
+        <v>530</v>
       </c>
       <c r="F22" s="2" t="s">
         <v>79</v>
@@ -7135,10 +7090,10 @@
         <v>73</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>535</v>
+        <v>531</v>
       </c>
       <c r="J22" s="2" t="s">
         <v>34</v>
@@ -7152,13 +7107,13 @@
         <v>169</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>536</v>
+        <v>532</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>536</v>
+        <v>532</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>537</v>
+        <v>533</v>
       </c>
       <c r="F23" s="2" t="s">
         <v>79</v>
@@ -7167,10 +7122,10 @@
         <v>111</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>538</v>
+        <v>534</v>
       </c>
       <c r="J23" s="2" t="s">
         <v>34</v>
@@ -7184,25 +7139,25 @@
         <v>173</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>539</v>
+        <v>535</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>539</v>
+        <v>535</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>540</v>
+        <v>536</v>
       </c>
       <c r="F24" s="2" t="s">
         <v>79</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>541</v>
+        <v>537</v>
       </c>
       <c r="J24" s="2" t="s">
         <v>34</v>
@@ -7216,13 +7171,13 @@
         <v>177</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>542</v>
+        <v>538</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>542</v>
+        <v>538</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>543</v>
+        <v>539</v>
       </c>
       <c r="F25" s="2" t="s">
         <v>79</v>
@@ -7231,10 +7186,10 @@
         <v>73</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>544</v>
+        <v>540</v>
       </c>
       <c r="J25" s="2" t="s">
         <v>34</v>
@@ -7248,13 +7203,13 @@
         <v>182</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>545</v>
+        <v>541</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>545</v>
+        <v>541</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>546</v>
+        <v>542</v>
       </c>
       <c r="F26" s="2" t="s">
         <v>79</v>
@@ -7263,10 +7218,10 @@
         <v>111</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>547</v>
+        <v>543</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>548</v>
+        <v>544</v>
       </c>
       <c r="J26" s="2" t="s">
         <v>34</v>
@@ -7280,25 +7235,25 @@
         <v>186</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>549</v>
+        <v>545</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>549</v>
+        <v>545</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>550</v>
+        <v>546</v>
       </c>
       <c r="F27" s="2" t="s">
         <v>79</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>80</v>
+        <v>374</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>551</v>
+        <v>370</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>552</v>
+        <v>547</v>
       </c>
       <c r="J27" s="2" t="s">
         <v>34</v>
@@ -7312,25 +7267,25 @@
         <v>190</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>553</v>
+        <v>548</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>553</v>
+        <v>548</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>554</v>
+        <v>549</v>
       </c>
       <c r="F28" s="2" t="s">
         <v>79</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>378</v>
+        <v>80</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>374</v>
+        <v>550</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>555</v>
+        <v>551</v>
       </c>
       <c r="J28" s="2" t="s">
         <v>34</v>
@@ -7344,25 +7299,25 @@
         <v>194</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>556</v>
+        <v>552</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>556</v>
+        <v>552</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>557</v>
+        <v>553</v>
       </c>
       <c r="F29" s="2" t="s">
         <v>79</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>558</v>
+        <v>554</v>
       </c>
       <c r="I29" s="2" t="s">
-        <v>559</v>
+        <v>555</v>
       </c>
       <c r="J29" s="2" t="s">
         <v>34</v>

</xml_diff>